<commit_message>
verbeterde opzet van ontstaan.md
</commit_message>
<xml_diff>
--- a/doc/regels.xlsx
+++ b/doc/regels.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cool\COOLbackend\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0480E2B3-CF06-4DED-A52B-9F2B2184FEC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DEDD232-B3C3-409F-A37E-98A571C9393B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{55F92E86-A93A-45F8-82E9-A9C823D47708}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
   <si>
     <t>Server</t>
   </si>
@@ -204,6 +204,12 @@
   </si>
   <si>
     <t>api-endpoints</t>
+  </si>
+  <si>
+    <t>server.js</t>
+  </si>
+  <si>
+    <t>0.8.67</t>
   </si>
 </sst>
 </file>
@@ -601,21 +607,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{040BBC20-915C-4A99-933E-A413CC83A31C}">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="6.59765625" customWidth="1"/>
+    <col min="3" max="3" width="7.53125" customWidth="1"/>
+    <col min="4" max="4" width="3.06640625" customWidth="1"/>
+    <col min="5" max="5" width="6.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.65">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.65">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="E1" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -623,11 +636,12 @@
         <v>11</v>
       </c>
       <c r="C2" s="3">
-        <f t="shared" ref="C2:C57" si="0">ROUND(B2/B$61,3)</f>
+        <f t="shared" ref="C2:C58" si="0">ROUND(B2/B$62,3)</f>
         <v>1E-3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -638,8 +652,9 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -650,8 +665,9 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -662,8 +678,9 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D5" s="3"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -674,8 +691,9 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D6" s="3"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -686,8 +704,9 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D7" s="3"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -698,8 +717,9 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D8" s="3"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -710,8 +730,9 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D9" s="3"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -723,8 +744,9 @@
         <f t="shared" si="0"/>
         <v>0.10100000000000001</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -733,10 +755,11 @@
       </c>
       <c r="C11" s="3">
         <f t="shared" si="0"/>
-        <v>0.19700000000000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+        <v>0.19900000000000001</v>
+      </c>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="12" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -747,30 +770,39 @@
         <f t="shared" si="0"/>
         <v>4.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="D12" s="3"/>
+    </row>
+    <row r="13" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B13" s="2">
         <f>SUM(B2:B12)</f>
         <v>2768</v>
       </c>
       <c r="C13" s="3">
         <f t="shared" si="0"/>
-        <v>0.312</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+        <v>0.315</v>
+      </c>
+      <c r="D13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="C14" s="3"/>
-    </row>
-    <row r="15" spans="1:3" ht="21" x14ac:dyDescent="0.65">
+      <c r="D14" s="3"/>
+    </row>
+    <row r="15" spans="1:5" ht="21" x14ac:dyDescent="0.65">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>2</v>
+      <c r="B15" s="4" t="str">
+        <f>B1</f>
+        <v>regels</v>
       </c>
       <c r="C15" s="3"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D15" s="3"/>
+      <c r="E15" s="4" t="str">
+        <f>E1</f>
+        <v>0.8.67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -781,8 +813,9 @@
         <f t="shared" si="0"/>
         <v>5.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D16" s="3"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -793,8 +826,9 @@
         <f t="shared" si="0"/>
         <v>4.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D17" s="3"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -805,8 +839,9 @@
         <f t="shared" si="0"/>
         <v>4.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -817,8 +852,9 @@
         <f t="shared" si="0"/>
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -829,8 +865,9 @@
         <f t="shared" si="0"/>
         <v>5.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -841,8 +878,9 @@
         <f t="shared" si="0"/>
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -853,8 +891,9 @@
         <f t="shared" si="0"/>
         <v>5.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D22" s="3"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -865,8 +904,9 @@
         <f t="shared" si="0"/>
         <v>4.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D23" s="3"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -877,8 +917,9 @@
         <f t="shared" si="0"/>
         <v>6.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D24" s="3"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -889,8 +930,9 @@
         <f t="shared" si="0"/>
         <v>3.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D25" s="3"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -901,8 +943,9 @@
         <f t="shared" si="0"/>
         <v>4.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D26" s="3"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -913,8 +956,9 @@
         <f t="shared" si="0"/>
         <v>8.0000000000000002E-3</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D27" s="3"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -925,8 +969,9 @@
         <f t="shared" si="0"/>
         <v>4.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -937,8 +982,9 @@
         <f t="shared" si="0"/>
         <v>3.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D29" s="3"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -949,8 +995,9 @@
         <f t="shared" si="0"/>
         <v>5.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D30" s="3"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -961,8 +1008,9 @@
         <f t="shared" si="0"/>
         <v>3.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D31" s="3"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -973,8 +1021,9 @@
         <f t="shared" si="0"/>
         <v>4.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D32" s="3"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -985,8 +1034,9 @@
         <f t="shared" si="0"/>
         <v>7.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D33" s="3"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -997,8 +1047,9 @@
         <f t="shared" si="0"/>
         <v>2E-3</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D34" s="3"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -1009,8 +1060,9 @@
         <f t="shared" si="0"/>
         <v>1.7000000000000001E-2</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D35" s="3"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1021,8 +1073,9 @@
         <f t="shared" si="0"/>
         <v>0.02</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D36" s="3"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -1033,8 +1086,9 @@
         <f t="shared" si="0"/>
         <v>1.4E-2</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D37" s="3"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -1045,8 +1099,9 @@
         <f t="shared" si="0"/>
         <v>8.9999999999999993E-3</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D38" s="3"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -1057,8 +1112,9 @@
         <f t="shared" si="0"/>
         <v>2.3E-2</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D39" s="3"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>48</v>
       </c>
@@ -1069,8 +1125,9 @@
         <f t="shared" si="0"/>
         <v>0.10100000000000001</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D40" s="3"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>38</v>
       </c>
@@ -1081,8 +1138,9 @@
         <f t="shared" si="0"/>
         <v>3.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D41" s="3"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>49</v>
       </c>
@@ -1093,8 +1151,9 @@
         <f t="shared" si="0"/>
         <v>2.4E-2</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D42" s="3"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>39</v>
       </c>
@@ -1105,8 +1164,9 @@
         <f t="shared" si="0"/>
         <v>0.05</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D43" s="3"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>40</v>
       </c>
@@ -1115,22 +1175,24 @@
       </c>
       <c r="C44" s="3">
         <f t="shared" si="0"/>
-        <v>1.9E-2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.45">
+        <v>0.02</v>
+      </c>
+      <c r="D44" s="3"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>41</v>
       </c>
       <c r="B45">
-        <v>523</v>
+        <v>288</v>
       </c>
       <c r="C45" s="3">
         <f t="shared" si="0"/>
-        <v>5.8999999999999997E-2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="D45" s="3"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>42</v>
       </c>
@@ -1141,8 +1203,9 @@
         <f t="shared" si="0"/>
         <v>2.1000000000000001E-2</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D46" s="3"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>43</v>
       </c>
@@ -1153,8 +1216,9 @@
         <f t="shared" si="0"/>
         <v>1.2E-2</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D47" s="3"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>50</v>
       </c>
@@ -1163,10 +1227,11 @@
       </c>
       <c r="C48" s="3">
         <f t="shared" si="0"/>
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="D48" s="3"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>6</v>
       </c>
@@ -1177,140 +1242,179 @@
         <f t="shared" si="0"/>
         <v>1.2E-2</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D49" s="3"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
+        <v>56</v>
+      </c>
+      <c r="B50">
+        <v>162</v>
+      </c>
+      <c r="C50" s="3">
+        <f t="shared" si="0"/>
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="D50" s="3"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
         <v>44</v>
       </c>
-      <c r="B50">
+      <c r="B51">
         <v>56</v>
       </c>
-      <c r="C50" s="3">
+      <c r="C51" s="3">
         <f t="shared" si="0"/>
         <v>6.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A51" t="s">
+      <c r="D51" s="3"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A52" t="s">
         <v>7</v>
       </c>
-      <c r="B51">
+      <c r="B52">
         <v>157</v>
       </c>
-      <c r="C51" s="3">
+      <c r="C52" s="3">
         <f t="shared" si="0"/>
         <v>1.7999999999999999E-2</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
+      <c r="D52" s="3"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
         <v>45</v>
       </c>
-      <c r="B52">
+      <c r="B53">
         <v>76</v>
       </c>
-      <c r="C52" s="3">
+      <c r="C53" s="3">
         <f t="shared" si="0"/>
         <v>8.9999999999999993E-3</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A53" t="s">
+      <c r="D53" s="3"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A54" t="s">
         <v>8</v>
       </c>
-      <c r="B53">
+      <c r="B54">
         <v>54</v>
       </c>
-      <c r="C53" s="3">
+      <c r="C54" s="3">
         <f t="shared" si="0"/>
         <v>6.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A54" t="s">
+      <c r="D54" s="3"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A55" t="s">
         <v>46</v>
       </c>
-      <c r="B54">
+      <c r="B55">
         <v>217</v>
       </c>
-      <c r="C54" s="3">
-        <f t="shared" si="0"/>
-        <v>2.4E-2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A55" t="s">
+      <c r="C55" s="3">
+        <f t="shared" si="0"/>
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="D55" s="3"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A56" t="s">
         <v>47</v>
       </c>
-      <c r="B55">
+      <c r="B56">
         <v>21</v>
       </c>
-      <c r="C55" s="3">
+      <c r="C56" s="3">
         <f t="shared" si="0"/>
         <v>2E-3</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A56" t="s">
+      <c r="D56" s="3"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A57" t="s">
         <v>51</v>
       </c>
-      <c r="B56">
+      <c r="B57">
         <v>682</v>
       </c>
-      <c r="C56" s="3">
-        <f t="shared" si="0"/>
-        <v>7.6999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A57" t="s">
+      <c r="C57" s="3">
+        <f t="shared" si="0"/>
+        <v>7.8E-2</v>
+      </c>
+      <c r="D57" s="3"/>
+    </row>
+    <row r="58" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A58" t="s">
         <v>52</v>
       </c>
-      <c r="B57">
+      <c r="B58">
         <v>301</v>
       </c>
-      <c r="C57" s="3">
+      <c r="C58" s="3">
         <f t="shared" si="0"/>
         <v>3.4000000000000002E-2</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="B58" s="2">
-        <f>SUM(B16:B57)</f>
-        <v>6104</v>
-      </c>
-      <c r="C58" s="3">
-        <f>ROUND(B58/B$61,3)</f>
-        <v>0.68799999999999994</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A60" t="s">
+      <c r="D58" s="3"/>
+    </row>
+    <row r="59" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="B59" s="2">
+        <f>SUM(B16:B58)</f>
+        <v>6031</v>
+      </c>
+      <c r="C59" s="3">
+        <f>ROUND(B59/B$62,3)</f>
+        <v>0.68500000000000005</v>
+      </c>
+      <c r="D59" s="3"/>
+      <c r="E59" s="2">
+        <f>SUM(E16:E58)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A61" t="s">
         <v>53</v>
       </c>
-      <c r="B60">
+      <c r="B61">
         <f>B13</f>
         <v>2768</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A61" t="s">
+      <c r="E61">
+        <f>E13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A62" t="s">
         <v>54</v>
       </c>
-      <c r="B61" s="2">
-        <f>B58+B60</f>
-        <v>8872</v>
-      </c>
-      <c r="C61" s="3">
-        <f>ROUND(B61/B$61,3)</f>
+      <c r="B62" s="2">
+        <f>B59+B61</f>
+        <v>8799</v>
+      </c>
+      <c r="C62" s="3">
+        <f>ROUND(B62/B$62,3)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A63" t="s">
+      <c r="D62" s="3"/>
+      <c r="E62" s="2">
+        <f>E59+E61</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A64" t="s">
         <v>55</v>
       </c>
-      <c r="B63">
+      <c r="B64">
+        <v>64</v>
+      </c>
+      <c r="E64">
         <v>64</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ontstaan.md is weer compleet
</commit_message>
<xml_diff>
--- a/doc/regels.xlsx
+++ b/doc/regels.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cool\COOLbackend\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DEDD232-B3C3-409F-A37E-98A571C9393B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE192018-27F0-4E5D-A6C9-333A80CA8D02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{55F92E86-A93A-45F8-82E9-A9C823D47708}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
   <si>
     <t>Server</t>
   </si>
@@ -209,7 +209,16 @@
     <t>server.js</t>
   </si>
   <si>
-    <t>0.8.67</t>
+    <t>0.8.66</t>
+  </si>
+  <si>
+    <t>Linux</t>
+  </si>
+  <si>
+    <t>wc -l *.js</t>
+  </si>
+  <si>
+    <t>browser</t>
   </si>
 </sst>
 </file>
@@ -607,17 +616,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{040BBC20-915C-4A99-933E-A413CC83A31C}">
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="6.59765625" customWidth="1"/>
-    <col min="3" max="3" width="7.53125" customWidth="1"/>
+    <col min="2" max="3" width="7.59765625" customWidth="1"/>
     <col min="4" max="4" width="3.06640625" customWidth="1"/>
-    <col min="5" max="5" width="6.59765625" customWidth="1"/>
+    <col min="5" max="6" width="7.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.65">
+    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.65">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -628,7 +636,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -636,12 +644,19 @@
         <v>11</v>
       </c>
       <c r="C2" s="3">
-        <f t="shared" ref="C2:C58" si="0">ROUND(B2/B$62,3)</f>
+        <f t="shared" ref="C2:C58" si="0">ROUND(B2/B$63,3)</f>
         <v>1E-3</v>
       </c>
       <c r="D2" s="3"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2" s="3">
+        <f t="shared" ref="F2:F58" si="1">ROUND(E2/E$63,3)</f>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -653,8 +668,15 @@
         <v>1E-3</v>
       </c>
       <c r="D3" s="3"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3">
+        <f t="shared" si="1"/>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -666,8 +688,15 @@
         <v>1E-3</v>
       </c>
       <c r="D4" s="3"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E4">
+        <v>10</v>
+      </c>
+      <c r="F4" s="3">
+        <f t="shared" si="1"/>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -679,8 +708,15 @@
         <v>1E-3</v>
       </c>
       <c r="D5" s="3"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="F5" s="3">
+        <f t="shared" si="1"/>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -692,8 +728,15 @@
         <v>1E-3</v>
       </c>
       <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6" s="3">
+        <f t="shared" si="1"/>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -705,8 +748,15 @@
         <v>1E-3</v>
       </c>
       <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E7">
+        <v>10</v>
+      </c>
+      <c r="F7" s="3">
+        <f t="shared" si="1"/>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -718,8 +768,15 @@
         <v>1E-3</v>
       </c>
       <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E8">
+        <v>10</v>
+      </c>
+      <c r="F8" s="3">
+        <f t="shared" si="1"/>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -731,8 +788,15 @@
         <v>1E-3</v>
       </c>
       <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E9">
+        <v>10</v>
+      </c>
+      <c r="F9" s="3">
+        <f t="shared" si="1"/>
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -745,8 +809,16 @@
         <v>0.10100000000000001</v>
       </c>
       <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E10">
+        <f>E40</f>
+        <v>781</v>
+      </c>
+      <c r="F10" s="3">
+        <f t="shared" si="1"/>
+        <v>9.4E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -758,8 +830,15 @@
         <v>0.19900000000000001</v>
       </c>
       <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="E11">
+        <v>1718</v>
+      </c>
+      <c r="F11" s="3">
+        <f t="shared" si="1"/>
+        <v>0.20599999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -771,8 +850,15 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="E12">
+        <v>37</v>
+      </c>
+      <c r="F12" s="3">
+        <f t="shared" si="1"/>
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B13" s="2">
         <f>SUM(B2:B12)</f>
         <v>2768</v>
@@ -782,12 +868,21 @@
         <v>0.315</v>
       </c>
       <c r="D13" s="3"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E13" s="2">
+        <f>SUM(E2:E12)</f>
+        <v>2616</v>
+      </c>
+      <c r="F13" s="3">
+        <f t="shared" si="1"/>
+        <v>0.314</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
-    </row>
-    <row r="15" spans="1:5" ht="21" x14ac:dyDescent="0.65">
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:6" ht="21" x14ac:dyDescent="0.65">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -799,10 +894,11 @@
       <c r="D15" s="3"/>
       <c r="E15" s="4" t="str">
         <f>E1</f>
-        <v>0.8.67</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+        <v>0.8.66</v>
+      </c>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -814,8 +910,15 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="D16" s="3"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E16">
+        <v>40</v>
+      </c>
+      <c r="F16" s="3">
+        <f t="shared" ref="F16:F65" si="2">ROUND(E16/E$63,3)</f>
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -827,8 +930,15 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="D17" s="3"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E17">
+        <v>31</v>
+      </c>
+      <c r="F17" s="3">
+        <f t="shared" si="2"/>
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -840,8 +950,15 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="D18" s="3"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E18">
+        <v>33</v>
+      </c>
+      <c r="F18" s="3">
+        <f t="shared" si="2"/>
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -853,8 +970,15 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="D19" s="3"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E19">
+        <v>64</v>
+      </c>
+      <c r="F19" s="3">
+        <f t="shared" si="2"/>
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -866,8 +990,15 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="D20" s="3"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E20">
+        <v>46</v>
+      </c>
+      <c r="F20" s="3">
+        <f t="shared" si="2"/>
+        <v>6.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -879,8 +1010,15 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="D21" s="3"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E21">
+        <v>62</v>
+      </c>
+      <c r="F21" s="3">
+        <f t="shared" si="2"/>
+        <v>7.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -892,8 +1030,15 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="D22" s="3"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E22">
+        <v>39</v>
+      </c>
+      <c r="F22" s="3">
+        <f t="shared" si="2"/>
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -905,8 +1050,15 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="D23" s="3"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E23">
+        <v>36</v>
+      </c>
+      <c r="F23" s="3">
+        <f t="shared" si="2"/>
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -918,8 +1070,15 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="D24" s="3"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E24">
+        <v>52</v>
+      </c>
+      <c r="F24" s="3">
+        <f t="shared" si="2"/>
+        <v>6.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -931,8 +1090,15 @@
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="D25" s="3"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E25">
+        <v>22</v>
+      </c>
+      <c r="F25" s="3">
+        <f t="shared" si="2"/>
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -944,8 +1110,15 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="D26" s="3"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E26">
+        <v>35</v>
+      </c>
+      <c r="F26" s="3">
+        <f t="shared" si="2"/>
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -957,8 +1130,15 @@
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="D27" s="3"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E27">
+        <v>71</v>
+      </c>
+      <c r="F27" s="3">
+        <f t="shared" si="2"/>
+        <v>8.9999999999999993E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -970,8 +1150,15 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="D28" s="3"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E28">
+        <v>31</v>
+      </c>
+      <c r="F28" s="3">
+        <f t="shared" si="2"/>
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -983,8 +1170,15 @@
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="D29" s="3"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E29">
+        <v>26</v>
+      </c>
+      <c r="F29" s="3">
+        <f t="shared" si="2"/>
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -996,8 +1190,15 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="D30" s="3"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E30">
+        <v>47</v>
+      </c>
+      <c r="F30" s="3">
+        <f t="shared" si="2"/>
+        <v>6.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -1009,8 +1210,15 @@
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="D31" s="3"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E31">
+        <v>23</v>
+      </c>
+      <c r="F31" s="3">
+        <f t="shared" si="2"/>
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -1022,8 +1230,15 @@
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="D32" s="3"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E32">
+        <v>36</v>
+      </c>
+      <c r="F32" s="3">
+        <f t="shared" si="2"/>
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -1035,8 +1250,15 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="D33" s="3"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E33">
+        <v>60</v>
+      </c>
+      <c r="F33" s="3">
+        <f t="shared" si="2"/>
+        <v>7.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -1048,8 +1270,15 @@
         <v>2E-3</v>
       </c>
       <c r="D34" s="3"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E34">
+        <v>14</v>
+      </c>
+      <c r="F34" s="3">
+        <f t="shared" si="2"/>
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -1061,8 +1290,15 @@
         <v>1.7000000000000001E-2</v>
       </c>
       <c r="D35" s="3"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E35">
+        <v>147</v>
+      </c>
+      <c r="F35" s="3">
+        <f t="shared" si="2"/>
+        <v>1.7999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1074,8 +1310,15 @@
         <v>0.02</v>
       </c>
       <c r="D36" s="3"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E36">
+        <v>175</v>
+      </c>
+      <c r="F36" s="3">
+        <f t="shared" si="2"/>
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -1087,8 +1330,15 @@
         <v>1.4E-2</v>
       </c>
       <c r="D37" s="3"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E37">
+        <v>122</v>
+      </c>
+      <c r="F37" s="3">
+        <f t="shared" si="2"/>
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -1100,8 +1350,15 @@
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="D38" s="3"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E38">
+        <v>77</v>
+      </c>
+      <c r="F38" s="3">
+        <f t="shared" si="2"/>
+        <v>8.9999999999999993E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -1113,8 +1370,15 @@
         <v>2.3E-2</v>
       </c>
       <c r="D39" s="3"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E39">
+        <v>192</v>
+      </c>
+      <c r="F39" s="3">
+        <f t="shared" si="2"/>
+        <v>2.3E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>48</v>
       </c>
@@ -1126,8 +1390,15 @@
         <v>0.10100000000000001</v>
       </c>
       <c r="D40" s="3"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E40">
+        <v>781</v>
+      </c>
+      <c r="F40" s="3">
+        <f t="shared" si="2"/>
+        <v>9.4E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>38</v>
       </c>
@@ -1139,8 +1410,15 @@
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="D41" s="3"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E41">
+        <v>29</v>
+      </c>
+      <c r="F41" s="3">
+        <f t="shared" si="2"/>
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>49</v>
       </c>
@@ -1152,8 +1430,15 @@
         <v>2.4E-2</v>
       </c>
       <c r="D42" s="3"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E42">
+        <v>211</v>
+      </c>
+      <c r="F42" s="3">
+        <f t="shared" si="2"/>
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>39</v>
       </c>
@@ -1165,8 +1450,15 @@
         <v>0.05</v>
       </c>
       <c r="D43" s="3"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E43">
+        <v>439</v>
+      </c>
+      <c r="F43" s="3">
+        <f t="shared" si="2"/>
+        <v>5.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>40</v>
       </c>
@@ -1178,8 +1470,15 @@
         <v>0.02</v>
       </c>
       <c r="D44" s="3"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E44">
+        <v>171</v>
+      </c>
+      <c r="F44" s="3">
+        <f t="shared" si="2"/>
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>41</v>
       </c>
@@ -1191,8 +1490,15 @@
         <v>3.3000000000000002E-2</v>
       </c>
       <c r="D45" s="3"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E45">
+        <v>424</v>
+      </c>
+      <c r="F45" s="3">
+        <f t="shared" si="2"/>
+        <v>5.0999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>42</v>
       </c>
@@ -1204,8 +1510,15 @@
         <v>2.1000000000000001E-2</v>
       </c>
       <c r="D46" s="3"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E46">
+        <v>101</v>
+      </c>
+      <c r="F46" s="3">
+        <f t="shared" si="2"/>
+        <v>1.2E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>43</v>
       </c>
@@ -1217,8 +1530,15 @@
         <v>1.2E-2</v>
       </c>
       <c r="D47" s="3"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E47">
+        <v>108</v>
+      </c>
+      <c r="F47" s="3">
+        <f t="shared" si="2"/>
+        <v>1.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>50</v>
       </c>
@@ -1230,8 +1550,15 @@
         <v>4.1000000000000002E-2</v>
       </c>
       <c r="D48" s="3"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E48">
+        <v>307</v>
+      </c>
+      <c r="F48" s="3">
+        <f t="shared" si="2"/>
+        <v>3.6999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>6</v>
       </c>
@@ -1243,8 +1570,15 @@
         <v>1.2E-2</v>
       </c>
       <c r="D49" s="3"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E49">
+        <v>104</v>
+      </c>
+      <c r="F49" s="3">
+        <f t="shared" si="2"/>
+        <v>1.2E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -1256,8 +1590,15 @@
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="D50" s="3"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>44</v>
       </c>
@@ -1269,8 +1610,15 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="D51" s="3"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E51">
+        <v>55</v>
+      </c>
+      <c r="F51" s="3">
+        <f t="shared" si="2"/>
+        <v>7.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>7</v>
       </c>
@@ -1282,8 +1630,15 @@
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="D52" s="3"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E52">
+        <v>164</v>
+      </c>
+      <c r="F52" s="3">
+        <f t="shared" si="2"/>
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>45</v>
       </c>
@@ -1295,8 +1650,15 @@
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="D53" s="3"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E53">
+        <v>69</v>
+      </c>
+      <c r="F53" s="3">
+        <f t="shared" si="2"/>
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>8</v>
       </c>
@@ -1308,8 +1670,15 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="D54" s="3"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E54">
+        <v>53</v>
+      </c>
+      <c r="F54" s="3">
+        <f t="shared" si="2"/>
+        <v>6.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>46</v>
       </c>
@@ -1321,8 +1690,15 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="D55" s="3"/>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E55">
+        <v>217</v>
+      </c>
+      <c r="F55" s="3">
+        <f t="shared" si="2"/>
+        <v>2.5999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>47</v>
       </c>
@@ -1334,8 +1710,15 @@
         <v>2E-3</v>
       </c>
       <c r="D56" s="3"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E56">
+        <v>20</v>
+      </c>
+      <c r="F56" s="3">
+        <f t="shared" si="2"/>
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>51</v>
       </c>
@@ -1347,8 +1730,15 @@
         <v>7.8E-2</v>
       </c>
       <c r="D57" s="3"/>
-    </row>
-    <row r="58" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="E57">
+        <v>681</v>
+      </c>
+      <c r="F57" s="3">
+        <f t="shared" si="2"/>
+        <v>8.2000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A58" t="s">
         <v>52</v>
       </c>
@@ -1360,23 +1750,34 @@
         <v>3.4000000000000002E-2</v>
       </c>
       <c r="D58" s="3"/>
-    </row>
-    <row r="59" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="E58">
+        <v>300</v>
+      </c>
+      <c r="F58" s="3">
+        <f t="shared" si="2"/>
+        <v>3.5999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B59" s="2">
         <f>SUM(B16:B58)</f>
         <v>6031</v>
       </c>
       <c r="C59" s="3">
-        <f>ROUND(B59/B$62,3)</f>
+        <f>ROUND(B59/B$63,3)</f>
         <v>0.68500000000000005</v>
       </c>
       <c r="D59" s="3"/>
       <c r="E59" s="2">
         <f>SUM(E16:E58)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+        <v>5715</v>
+      </c>
+      <c r="F59" s="3">
+        <f>ROUND(E59/E$63,3)</f>
+        <v>0.68600000000000005</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>53</v>
       </c>
@@ -1384,38 +1785,59 @@
         <f>B13</f>
         <v>2768</v>
       </c>
-      <c r="E61">
+    </row>
+    <row r="62" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A62" t="s">
+        <v>60</v>
+      </c>
+      <c r="B62">
+        <f>B59</f>
+        <v>6031</v>
+      </c>
+      <c r="E62">
         <f>E13</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A62" t="s">
+        <v>2616</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A63" t="s">
         <v>54</v>
       </c>
-      <c r="B62" s="2">
-        <f>B59+B61</f>
+      <c r="B63" s="2">
+        <f>B13+B59</f>
         <v>8799</v>
       </c>
-      <c r="C62" s="3">
-        <f>ROUND(B62/B$62,3)</f>
+      <c r="C63" s="3">
+        <f>ROUND(B63/B$63,3)</f>
         <v>1</v>
       </c>
-      <c r="D62" s="3"/>
-      <c r="E62" s="2">
-        <f>E59+E61</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A64" t="s">
+      <c r="D63" s="3"/>
+      <c r="E63" s="2">
+        <f>E59+E62</f>
+        <v>8331</v>
+      </c>
+      <c r="F63" s="3">
+        <f>ROUND(E63/E$63,3)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A65" t="s">
         <v>55</v>
       </c>
-      <c r="B64">
+      <c r="B65">
         <v>64</v>
       </c>
-      <c r="E64">
-        <v>64</v>
+      <c r="E65">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="21" x14ac:dyDescent="0.65">
+      <c r="A68" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B68" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>